<commit_message>
Add info & links
</commit_message>
<xml_diff>
--- a/easy_20260228.xlsx
+++ b/easy_20260228.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5102170ae7533958/Documents/Programmation/rust/97_codingame/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F777DCE491E04430478DD1A7E0D8F6C360A1E00F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84E95069-B9AC-425B-98CE-F48284E2B1EA}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_F777DCE491E04430478DD1A7E0D8F6C360A1E00F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2913872-1025-4CF8-B44A-333CED27A1DA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="309">
   <si>
     <t>titre</t>
   </si>
@@ -2085,7 +2085,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>244</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>168</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>167</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>141</v>
       </c>
@@ -2129,16 +2129,21 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>195</v>
       </c>
       <c r="B69">
         <v>2078</v>
       </c>
-      <c r="C69" s="1"/>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C69" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D69" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>34</v>
       </c>
@@ -2149,7 +2154,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>43</v>
       </c>
@@ -2158,7 +2163,7 @@
       </c>
       <c r="C71" s="1"/>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>224</v>
       </c>
@@ -2169,7 +2174,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -2180,7 +2185,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>233</v>
       </c>
@@ -2191,7 +2196,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>158</v>
       </c>
@@ -2202,7 +2207,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>70</v>
       </c>
@@ -2213,7 +2218,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>176</v>
       </c>
@@ -2224,7 +2229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>179</v>
       </c>
@@ -2233,7 +2238,7 @@
       </c>
       <c r="C78" s="1"/>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>101</v>
       </c>
@@ -2244,7 +2249,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>187</v>
       </c>

</xml_diff>